<commit_message>
Remove campos de cargo e setor do componente de participantes e diálogos relacionados, simplificando a interface e a lógica de manipulação de dados. Atualiza a importação de participantes para incluir cargo e setor diretamente das planilhas, melhorando a experiência do usuário ao gerenciar informações de participantes.
</commit_message>
<xml_diff>
--- a/src/assets/templates/Modelo_Avaliacao_360.xlsx
+++ b/src/assets/templates/Modelo_Avaliacao_360.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
   <si>
     <t xml:space="preserve">Formulário de Solicitação - Avaliação 360°</t>
   </si>
@@ -29,9 +29,6 @@
   </si>
   <si>
     <t xml:space="preserve">Se você tiver alguma dúvida, entre em contato por e-mail.					</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indicação de Avaliadores por categoria </t>
   </si>
   <si>
     <t xml:space="preserve">Exemplo:   
@@ -44,9 +41,6 @@
     <t xml:space="preserve">Categoria</t>
   </si>
   <si>
-    <t xml:space="preserve">Número mínimo</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Número Ideal </t>
   </si>
   <si>
@@ -93,9 +87,6 @@
   </si>
   <si>
     <t xml:space="preserve">Nome e Sobrenome</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cargo/Setor</t>
   </si>
 </sst>
 </file>
@@ -105,7 +96,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -182,13 +173,6 @@
     <font>
       <b val="true"/>
       <sz val="9"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="9"/>
       <color rgb="FFEE0000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -465,7 +449,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -554,10 +538,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -578,27 +558,23 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -718,9 +694,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1591200</xdr:colOff>
+      <xdr:colOff>1590840</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>856800</xdr:rowOff>
+      <xdr:rowOff>856440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -735,7 +711,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="431280" y="101880"/>
-          <a:ext cx="1504080" cy="888120"/>
+          <a:ext cx="1503720" cy="887760"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -936,9 +912,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="55.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="49.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="2.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="2.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="10.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -951,7 +927,6 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="3"/>
@@ -959,8 +934,7 @@
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="5"/>
+      <c r="G3" s="5"/>
     </row>
     <row r="4" s="6" customFormat="true" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="7"/>
@@ -970,8 +944,8 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
       <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="0"/>
     </row>
     <row r="5" s="6" customFormat="true" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="7"/>
@@ -981,8 +955,8 @@
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="0"/>
     </row>
     <row r="6" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="11"/>
@@ -990,175 +964,149 @@
       <c r="D6" s="12"/>
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="13"/>
+      <c r="G6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="11"/>
       <c r="C7" s="14"/>
       <c r="D7" s="14"/>
       <c r="E7" s="14"/>
-      <c r="F7" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="G7" s="15"/>
-      <c r="H7" s="13"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="13"/>
     </row>
     <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="11"/>
       <c r="C8" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="E8" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="16" t="s">
+      <c r="F8" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="F8" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="H8" s="13"/>
+      <c r="G8" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="11"/>
       <c r="C9" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="19" t="s">
         <v>9</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="E9" s="19" t="s">
-        <v>11</v>
       </c>
       <c r="F9" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="13"/>
+      <c r="G9" s="13"/>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="11"/>
       <c r="C10" s="19" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>13</v>
+        <v>8</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>11</v>
       </c>
       <c r="F10" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="H10" s="13"/>
+      <c r="G10" s="13"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="11"/>
       <c r="C11" s="19" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>15</v>
+        <v>8</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>13</v>
       </c>
       <c r="F11" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="G11" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="13"/>
+      <c r="G11" s="13"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="11"/>
       <c r="C12" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="D12" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="E12" s="23" t="s">
-        <v>17</v>
+        <v>14</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="22" t="s">
+        <v>15</v>
       </c>
       <c r="F12" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="G12" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="H12" s="13"/>
+      <c r="G12" s="13"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="11"/>
-      <c r="C13" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" s="26" t="s">
-        <v>19</v>
-      </c>
-      <c r="F13" s="27" t="n">
-        <v>2</v>
-      </c>
-      <c r="G13" s="28" t="n">
+      <c r="C13" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="13"/>
+      <c r="G13" s="13"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="11"/>
-      <c r="C14" s="29" t="s">
-        <v>20</v>
-      </c>
-      <c r="D14" s="29"/>
-      <c r="E14" s="30"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="13"/>
+      <c r="C14" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="27"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="13"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="11"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
-      <c r="F15" s="31"/>
-      <c r="G15" s="31"/>
-      <c r="H15" s="13"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="13"/>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="11"/>
-      <c r="C16" s="32" t="s">
-        <v>21</v>
-      </c>
-      <c r="D16" s="33"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="31"/>
-      <c r="G16" s="31"/>
-      <c r="H16" s="13"/>
+      <c r="C16" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="13"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="11"/>
-      <c r="C17" s="34" t="s">
-        <v>22</v>
-      </c>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="13"/>
+      <c r="C17" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="32"/>
+      <c r="G17" s="13"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="11"/>
@@ -1166,256 +1114,223 @@
       <c r="D18" s="12"/>
       <c r="E18" s="12"/>
       <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="13"/>
+      <c r="G18" s="13"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="11"/>
-      <c r="C19" s="35" t="s">
-        <v>23</v>
-      </c>
-      <c r="D19" s="35" t="s">
+      <c r="C19" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="D19" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="E19" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="E19" s="35" t="s">
-        <v>6</v>
-      </c>
-      <c r="F19" s="35" t="s">
-        <v>24</v>
-      </c>
-      <c r="G19" s="12"/>
-      <c r="H19" s="13"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="13"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="11"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="13"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="13"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="11"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="13"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="13"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="11"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="13"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="13"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="11"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="13"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="13"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="11"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="13"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="13"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="11"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="13"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="36"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="13"/>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="11"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="13"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="36"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="13"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="11"/>
-      <c r="C27" s="25"/>
-      <c r="D27" s="38"/>
-      <c r="E27" s="25"/>
-      <c r="F27" s="25"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="13"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="36"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="13"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="11"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="38"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="12"/>
-      <c r="H28" s="13"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="36"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="13"/>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="11"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="38"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="25"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="13"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="36"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="13"/>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="11"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="38"/>
-      <c r="E30" s="25"/>
-      <c r="F30" s="25"/>
-      <c r="G30" s="12"/>
-      <c r="H30" s="13"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="36"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="13"/>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="11"/>
-      <c r="C31" s="25"/>
-      <c r="D31" s="38"/>
-      <c r="E31" s="25"/>
-      <c r="F31" s="25"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="13"/>
+      <c r="C31" s="24"/>
+      <c r="D31" s="36"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="13"/>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="11"/>
-      <c r="C32" s="25"/>
-      <c r="D32" s="38"/>
-      <c r="E32" s="25"/>
-      <c r="F32" s="25"/>
-      <c r="G32" s="12"/>
-      <c r="H32" s="13"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="36"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="12"/>
+      <c r="G32" s="13"/>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="11"/>
-      <c r="C33" s="25"/>
-      <c r="D33" s="38"/>
-      <c r="E33" s="25"/>
-      <c r="F33" s="25"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="13"/>
+      <c r="C33" s="24"/>
+      <c r="D33" s="36"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="12"/>
+      <c r="G33" s="13"/>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="11"/>
-      <c r="C34" s="25"/>
-      <c r="D34" s="38"/>
-      <c r="E34" s="25"/>
-      <c r="F34" s="25"/>
-      <c r="G34" s="12"/>
-      <c r="H34" s="13"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="36"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="13"/>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="11"/>
-      <c r="C35" s="25"/>
-      <c r="D35" s="38"/>
-      <c r="E35" s="25"/>
-      <c r="F35" s="25"/>
-      <c r="G35" s="12"/>
-      <c r="H35" s="13"/>
+      <c r="C35" s="24"/>
+      <c r="D35" s="36"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="12"/>
+      <c r="G35" s="13"/>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="11"/>
-      <c r="C36" s="25"/>
-      <c r="D36" s="38"/>
-      <c r="E36" s="25"/>
-      <c r="F36" s="25"/>
-      <c r="G36" s="12"/>
-      <c r="H36" s="13"/>
+      <c r="C36" s="24"/>
+      <c r="D36" s="36"/>
+      <c r="E36" s="24"/>
+      <c r="F36" s="12"/>
+      <c r="G36" s="13"/>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="11"/>
-      <c r="C37" s="25"/>
-      <c r="D37" s="38"/>
-      <c r="E37" s="25"/>
-      <c r="F37" s="25"/>
-      <c r="G37" s="12"/>
-      <c r="H37" s="13"/>
+      <c r="C37" s="24"/>
+      <c r="D37" s="36"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="12"/>
+      <c r="G37" s="13"/>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="11"/>
-      <c r="C38" s="25"/>
-      <c r="D38" s="38"/>
-      <c r="E38" s="25"/>
-      <c r="F38" s="25"/>
-      <c r="G38" s="12"/>
-      <c r="H38" s="13"/>
+      <c r="C38" s="24"/>
+      <c r="D38" s="36"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="12"/>
+      <c r="G38" s="13"/>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="11"/>
-      <c r="C39" s="25"/>
-      <c r="D39" s="38"/>
-      <c r="E39" s="25"/>
-      <c r="F39" s="25"/>
-      <c r="G39" s="12"/>
-      <c r="H39" s="13"/>
+      <c r="C39" s="24"/>
+      <c r="D39" s="36"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="13"/>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="11"/>
-      <c r="C40" s="25"/>
-      <c r="D40" s="38"/>
-      <c r="E40" s="25"/>
-      <c r="F40" s="25"/>
-      <c r="G40" s="12"/>
-      <c r="H40" s="13"/>
+      <c r="C40" s="24"/>
+      <c r="D40" s="36"/>
+      <c r="E40" s="24"/>
+      <c r="F40" s="12"/>
+      <c r="G40" s="13"/>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="11"/>
-      <c r="C41" s="25"/>
-      <c r="D41" s="38"/>
-      <c r="E41" s="25"/>
-      <c r="F41" s="25"/>
-      <c r="G41" s="12"/>
-      <c r="H41" s="13"/>
+      <c r="C41" s="24"/>
+      <c r="D41" s="36"/>
+      <c r="E41" s="24"/>
+      <c r="F41" s="12"/>
+      <c r="G41" s="13"/>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="11"/>
-      <c r="C42" s="25"/>
-      <c r="D42" s="38"/>
-      <c r="E42" s="25"/>
-      <c r="F42" s="25"/>
-      <c r="G42" s="12"/>
-      <c r="H42" s="13"/>
+      <c r="C42" s="24"/>
+      <c r="D42" s="36"/>
+      <c r="E42" s="24"/>
+      <c r="F42" s="12"/>
+      <c r="G42" s="13"/>
     </row>
     <row r="43" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B43" s="39"/>
-      <c r="C43" s="40"/>
-      <c r="D43" s="40"/>
-      <c r="E43" s="40"/>
-      <c r="F43" s="40"/>
-      <c r="G43" s="40"/>
-      <c r="H43" s="41"/>
+      <c r="B43" s="37"/>
+      <c r="C43" s="38"/>
+      <c r="D43" s="38"/>
+      <c r="E43" s="38"/>
+      <c r="F43" s="38"/>
+      <c r="G43" s="39"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="F7:G7"/>
+  <mergeCells count="3">
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="C5:F5"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="1">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="E20:E42" type="list">
       <formula1>"Avaliado,Gestor,Par,Subordinado,Outros"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F20:F42" type="none">
-      <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>